<commit_message>
Add azure-core, azure-cosmos, and python-dotenv packages to project dependencies
- Introduced azure-core version 1.41.0 and azure-cosmos version 4.15.0 with their respective dependencies.
- Updated fiona-notebooks to include azure-cosmos and python-dotenv as dependencies.
- Added python-dotenv version 1.2.2 to manage environment variables.
</commit_message>
<xml_diff>
--- a/notebooks/usage-analytics/usage-analytics-export.xlsx
+++ b/notebooks/usage-analytics/usage-analytics-export.xlsx
@@ -178,12 +178,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Daily Summary'!$A$2:$A$24</f>
+              <f>'Daily Summary'!$A$2:$A$25</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Daily Summary'!$D$2:$D$24</f>
+              <f>'Daily Summary'!$D$2:$D$25</f>
             </numRef>
           </val>
         </ser>
@@ -290,12 +290,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Daily Summary'!$A$2:$A$24</f>
+              <f>'Daily Summary'!$A$2:$A$25</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Daily Summary'!$B$2:$B$24</f>
+              <f>'Daily Summary'!$B$2:$B$25</f>
             </numRef>
           </val>
         </ser>
@@ -409,12 +409,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Daily Summary'!$A$2:$A$24</f>
+              <f>'Daily Summary'!$A$2:$A$25</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Daily Summary'!$F$2:$F$24</f>
+              <f>'Daily Summary'!$F$2:$F$25</f>
             </numRef>
           </val>
         </ser>
@@ -1480,7 +1480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2101,6 +2101,31 @@
         <v>0</v>
       </c>
       <c r="G24" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>4</v>
+      </c>
+      <c r="C25" t="n">
+        <v>4</v>
+      </c>
+      <c r="D25" t="n">
+        <v>10</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2402,13 +2427,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C7" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D7" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
@@ -2429,7 +2454,7 @@
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="L7" t="n">
         <v>0</v>
@@ -3347,7 +3372,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3441,7 +3466,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C3" t="n">
         <v>1</v>
@@ -3456,14 +3481,14 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-05-15 12:09:59.063000-05:00</t>
+          <t>2026-05-19 10:11:42.270000-05:00</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>15.8</v>
+        <v>15</v>
       </c>
       <c r="H3" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4">
@@ -3533,107 +3558,107 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>UA7S95MU2</t>
+          <t>U07F6FFAVS9</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-04-20 11:16:29.778000-05:00</t>
+          <t>2026-04-16 17:47:16.683000-05:00</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-05-14 10:20:22.755000-05:00</t>
+          <t>2026-05-19 00:11:56.897000-05:00</t>
         </is>
       </c>
       <c r="G6" t="n">
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>8</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>U07F6FFAVS9</t>
+          <t>U07M86DHPDM</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D7" t="n">
         <v>0</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-04-16 17:47:16.683000-05:00</t>
+          <t>2026-04-30 17:28:38.894000-05:00</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-05-12 14:27:15.716000-05:00</t>
+          <t>2026-05-19 10:28:41.193000-05:00</t>
         </is>
       </c>
       <c r="G7" t="n">
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>2.3</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>UA0CMFN9G</t>
+          <t>UA7S95MU2</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D8" t="n">
         <v>0</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-04-16 17:48:32.236000-05:00</t>
+          <t>2026-04-20 11:16:29.778000-05:00</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-04-24 16:57:50.355000-05:00</t>
+          <t>2026-05-14 10:20:22.755000-05:00</t>
         </is>
       </c>
       <c r="G8" t="n">
         <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>2.3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>U056L1QEM1U</t>
+          <t>UA0CMFN9G</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C9" t="n">
         <v>3</v>
@@ -3643,19 +3668,19 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-05-07 11:35:31.688000-05:00</t>
+          <t>2026-04-16 17:48:32.236000-05:00</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-05-13 13:52:54.712000-05:00</t>
+          <t>2026-04-24 16:57:50.355000-05:00</t>
         </is>
       </c>
       <c r="G9" t="n">
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>1.7</v>
+        <v>2.3</v>
       </c>
     </row>
     <row r="10">
@@ -3693,75 +3718,75 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>U49PX6ZQD</t>
+          <t>U056L1QEM1U</t>
         </is>
       </c>
       <c r="B11" t="n">
         <v>5</v>
       </c>
       <c r="C11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D11" t="n">
         <v>0</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-04-27 10:47:36.948000-05:00</t>
+          <t>2026-05-07 11:35:31.688000-05:00</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-05-03 19:22:44.100000-05:00</t>
+          <t>2026-05-13 13:52:54.712000-05:00</t>
         </is>
       </c>
       <c r="G11" t="n">
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>1.2</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>U066VV53J1K</t>
+          <t>U49PX6ZQD</t>
         </is>
       </c>
       <c r="B12" t="n">
         <v>5</v>
       </c>
       <c r="C12" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D12" t="n">
         <v>0</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-04-27 09:08:11.813000-05:00</t>
+          <t>2026-04-27 10:47:36.948000-05:00</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-04-27 09:10:15.991000-05:00</t>
+          <t>2026-05-03 19:22:44.100000-05:00</t>
         </is>
       </c>
       <c r="G12" t="n">
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>5</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>U09BD5E9HS8</t>
+          <t>U066VV53J1K</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C13" t="n">
         <v>1</v>
@@ -3771,25 +3796,25 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-04-22 07:41:08.533000-05:00</t>
+          <t>2026-04-27 09:08:11.813000-05:00</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-04-30 11:26:50.866000-05:00</t>
+          <t>2026-04-27 09:10:15.991000-05:00</t>
         </is>
       </c>
       <c r="G13" t="n">
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>U050VK93A8Z</t>
+          <t>U0ARWT706RY</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -3803,12 +3828,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-04-23 16:32:29.897000-05:00</t>
+          <t>2026-05-04 16:26:50.927000-05:00</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-04-24 09:07:35.651000-05:00</t>
+          <t>2026-05-04 16:33:25.610000-05:00</t>
         </is>
       </c>
       <c r="G14" t="n">
@@ -3821,7 +3846,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>U04L3TY2091</t>
+          <t>U050VK93A8Z</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -3835,12 +3860,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-04-23 12:13:19.326000-05:00</t>
+          <t>2026-04-23 16:32:29.897000-05:00</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2026-04-23 16:52:53.980000-05:00</t>
+          <t>2026-04-24 09:07:35.651000-05:00</t>
         </is>
       </c>
       <c r="G15" t="n">
@@ -3853,39 +3878,39 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>U07M86DHPDM</t>
+          <t>U04L3TY2091</t>
         </is>
       </c>
       <c r="B16" t="n">
         <v>4</v>
       </c>
       <c r="C16" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D16" t="n">
         <v>0</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-04-30 17:28:38.894000-05:00</t>
+          <t>2026-04-23 12:13:19.326000-05:00</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026-05-11 11:47:25.046000-05:00</t>
+          <t>2026-04-23 16:52:53.980000-05:00</t>
         </is>
       </c>
       <c r="G16" t="n">
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>1.3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>U0ARWT706RY</t>
+          <t>U09BD5E9HS8</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -3899,12 +3924,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2026-05-04 16:26:50.927000-05:00</t>
+          <t>2026-04-22 07:41:08.533000-05:00</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-05-04 16:33:25.610000-05:00</t>
+          <t>2026-04-30 11:26:50.866000-05:00</t>
         </is>
       </c>
       <c r="G17" t="n">
@@ -3917,7 +3942,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>UGQ5YSCHL</t>
+          <t>U504VBR4P</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -3931,12 +3956,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2026-05-05 09:25:50.941000-05:00</t>
+          <t>2026-04-29 09:25:25.838000-05:00</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-05-05 09:27:15.949000-05:00</t>
+          <t>2026-04-29 09:27:41.836000-05:00</t>
         </is>
       </c>
       <c r="G18" t="n">
@@ -3949,7 +3974,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>U504VBR4P</t>
+          <t>UGQ5YSCHL</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -3963,12 +3988,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2026-04-29 09:25:25.838000-05:00</t>
+          <t>2026-05-05 09:25:50.941000-05:00</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-04-29 09:27:41.836000-05:00</t>
+          <t>2026-05-05 09:27:15.949000-05:00</t>
         </is>
       </c>
       <c r="G19" t="n">
@@ -4013,7 +4038,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>U0AB9PE1Z50</t>
+          <t>U09ELM4KDAN</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -4027,12 +4052,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-05-04 17:57:14.740000-05:00</t>
+          <t>2026-04-28 09:50:32.239000-05:00</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2026-05-04 17:57:14.740000-05:00</t>
+          <t>2026-04-28 09:50:32.239000-05:00</t>
         </is>
       </c>
       <c r="G21" t="n">
@@ -4077,7 +4102,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>U09ELM4KDAN</t>
+          <t>U0AB9PE1Z50</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -4091,12 +4116,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026-04-28 09:50:32.239000-05:00</t>
+          <t>2026-05-04 17:57:14.740000-05:00</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2026-04-28 09:50:32.239000-05:00</t>
+          <t>2026-05-04 17:57:14.740000-05:00</t>
         </is>
       </c>
       <c r="G23" t="n">
@@ -4135,6 +4160,38 @@
         <v>0</v>
       </c>
       <c r="H24" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>UNUB35QUQ</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>1</v>
+      </c>
+      <c r="C25" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>2026-05-19 16:10:24.128000-05:00</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>2026-05-19 16:10:24.128000-05:00</t>
+        </is>
+      </c>
+      <c r="G25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4176,7 +4233,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>216</v>
+        <v>226</v>
       </c>
     </row>
     <row r="3">
@@ -4186,7 +4243,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4">
@@ -4196,7 +4253,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>51</v>
+        <v>54</v>
       </c>
     </row>
     <row r="5">
@@ -4206,7 +4263,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3.2</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="6">

</xml_diff>